<commit_message>
Ajout de la page portfolio
</commit_message>
<xml_diff>
--- a/docs/Tableau-de-Synthese_Eren-Akyurek.xlsx
+++ b/docs/Tableau-de-Synthese_Eren-Akyurek.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\DEV\Portfolio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\DEV\Portfolio\portfolio\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{187E247D-6F53-4E59-98BA-2B018AD6CBE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{039FA131-7087-437B-9D8A-1BB236101F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -827,6 +827,54 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -844,54 +892,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1138,56 +1138,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27" t="s">
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="27"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31" t="s">
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="29"/>
-      <c r="H3" s="32"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="48"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="38"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="32"/>
       <c r="F4" s="2" t="s">
         <v>3</v>
       </c>
@@ -1199,22 +1199,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="41"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="38" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -1237,8 +1237,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="6" customFormat="1" ht="324.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="43"/>
-      <c r="B7" s="45"/>
+      <c r="A7" s="37"/>
+      <c r="B7" s="39"/>
       <c r="C7" s="22" t="s">
         <v>13</v>
       </c>
@@ -1294,16 +1294,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="6" customFormat="1" ht="17.649999999999999" x14ac:dyDescent="0.35">
-      <c r="A8" s="46" t="s">
+      <c r="A8" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="47"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="48"/>
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="42"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1352,10 +1352,9 @@
       <c r="E9" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="26" t="s">
+      <c r="G9" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="12"/>
       <c r="H9" s="26" t="s">
         <v>33</v>
       </c>
@@ -1835,16 +1834,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="6" customFormat="1" ht="17.649999999999999" x14ac:dyDescent="0.35">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="35"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="29"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -2218,16 +2217,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="6" customFormat="1" ht="17.649999999999999" x14ac:dyDescent="0.35">
-      <c r="A27" s="33" t="s">
+      <c r="A27" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="35"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="29"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2694,6 +2693,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="A4:E4"/>
@@ -2701,11 +2705,6 @@
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078738" right="0.19685039370078738" top="0.19685039370078738" bottom="0.19685039370078738" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -2714,12 +2713,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2885,15 +2881,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637C494D-8486-4767-AF03-4D2C0D7F3459}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DB7854F-1A38-41F5-B589-6778A38FBA89}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2917,10 +2917,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DB7854F-1A38-41F5-B589-6778A38FBA89}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{637C494D-8486-4767-AF03-4D2C0D7F3459}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>